<commit_message>
Flash in Bestelliste hinzugefügt
</commit_message>
<xml_diff>
--- a/Komponenten und Auslegung/Komponenten_aus_BOM_Vergleich.xlsx
+++ b/Komponenten und Auslegung/Komponenten_aus_BOM_Vergleich.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxec\Documents\Studium\4. Semester\Elektronische Produktentwicklung I\ELEK_Inv_Pen\Komponenten und Auslegung\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1ac616d471f04106/070_UNI/40_SS25/ELEKT/ELEK_Inv_Pen/Komponenten und Auslegung/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12FF9F2E-AB38-4E6E-8396-CC66151D87BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{12FF9F2E-AB38-4E6E-8396-CC66151D87BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{537E25FD-8518-4FD8-AC58-804C2335F457}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8387AABA-4531-477D-ACDD-FCEAA7839344}"/>
+    <workbookView minimized="1" xWindow="-11370" yWindow="7120" windowWidth="38660" windowHeight="11720" xr2:uid="{8387AABA-4531-477D-ACDD-FCEAA7839344}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1510,16 +1510,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B807A8D-C0E2-4C54-B251-D7A20DB38A6B}">
   <dimension ref="A1:G99"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
-    <col min="3" max="3" width="105.140625" customWidth="1"/>
-    <col min="4" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="7" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="29.453125" customWidth="1"/>
+    <col min="3" max="3" width="105.1796875" customWidth="1"/>
+    <col min="4" max="6" width="11.453125" customWidth="1"/>
+    <col min="7" max="7" width="26.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" ht="13">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3034,7 +3034,7 @@
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
     </row>
-    <row r="78" spans="1:7" ht="13.5" thickBot="1"/>
+    <row r="78" spans="1:7" ht="13" thickBot="1"/>
     <row r="79" spans="1:7">
       <c r="A79" s="4" t="s">
         <v>254</v>
@@ -3181,7 +3181,7 @@
       <c r="F87" s="2"/>
       <c r="G87" s="11"/>
     </row>
-    <row r="88" spans="1:7" ht="13.5" thickBot="1">
+    <row r="88" spans="1:7" ht="13" thickBot="1">
       <c r="A88" s="6"/>
       <c r="B88" s="12" t="s">
         <v>141</v>
@@ -3207,7 +3207,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="90" spans="1:7" ht="13.5" thickBot="1"/>
+    <row r="90" spans="1:7" ht="13" thickBot="1"/>
     <row r="91" spans="1:7">
       <c r="A91" s="4" t="s">
         <v>267</v>
@@ -3322,7 +3322,7 @@
       <c r="F97" s="2"/>
       <c r="G97" s="11"/>
     </row>
-    <row r="98" spans="1:7" ht="13.5" thickBot="1">
+    <row r="98" spans="1:7" ht="13" thickBot="1">
       <c r="A98" s="6"/>
       <c r="B98" s="12" t="s">
         <v>272</v>

</xml_diff>